<commit_message>
update cluster centers nber
</commit_message>
<xml_diff>
--- a/output/reports/cv_experiment_KNN_kmeans_classification.xlsx
+++ b/output/reports/cv_experiment_KNN_kmeans_classification.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,23 +491,23 @@
         <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1292474269866943</v>
+        <v>7.704506874084473</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9488473655426636</v>
+        <v>0.9078885893354798</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9805194805194806</v>
+        <v>0.9177215189873418</v>
       </c>
       <c r="G2" t="n">
-        <v>0.9745479449394199</v>
+        <v>0.9042719302588844</v>
       </c>
       <c r="H2" t="n">
-        <v>0.9994518468544443</v>
+        <v>0.9919666413299063</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>{'metric': 'manhattan', 'n_neighbors': 3, 'weights': 'distance'}</t>
+          <t>{'metric': 'manhattan', 'n_neighbors': 11, 'weights': 'distance'}</t>
         </is>
       </c>
     </row>
@@ -526,23 +526,93 @@
         <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1281981468200684</v>
+        <v>6.572227478027344</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9607823558176621</v>
+        <v>0.9100525295165802</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9805194805194806</v>
+        <v>0.9177215189873418</v>
       </c>
       <c r="G3" t="n">
-        <v>0.9745479449394199</v>
+        <v>0.9053970684014629</v>
       </c>
       <c r="H3" t="n">
-        <v>0.9994518468544443</v>
+        <v>0.992708122285623</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>{'metric': 'manhattan', 'n_neighbors': 3, 'weights': 'distance'}</t>
+          <t>{'metric': 'manhattan', 'n_neighbors': 15, 'weights': 'distance'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Classification</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>KNN</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D4" t="n">
+        <v>7.689805746078491</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.9133368902195146</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.9177215189873418</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.9053970684014629</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.992708122285623</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>{'metric': 'manhattan', 'n_neighbors': 15, 'weights': 'distance'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Classification</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>KNN</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>15</v>
+      </c>
+      <c r="D5" t="n">
+        <v>7.842351198196411</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.9129583933927897</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.9177215189873418</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.9053970684014629</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.992708122285623</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>{'metric': 'manhattan', 'n_neighbors': 15, 'weights': 'distance'}</t>
         </is>
       </c>
     </row>
@@ -557,7 +627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -622,23 +692,23 @@
         <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1292474269866943</v>
+        <v>7.704506874084473</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9488473655426636</v>
+        <v>0.9078885893354798</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9805194805194806</v>
+        <v>0.9177215189873418</v>
       </c>
       <c r="G2" t="n">
-        <v>0.9745479449394199</v>
+        <v>0.9042719302588844</v>
       </c>
       <c r="H2" t="n">
-        <v>0.9994518468544443</v>
+        <v>0.9919666413299063</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>{'metric': 'manhattan', 'n_neighbors': 3, 'weights': 'distance'}</t>
+          <t>{'metric': 'manhattan', 'n_neighbors': 11, 'weights': 'distance'}</t>
         </is>
       </c>
     </row>
@@ -657,23 +727,93 @@
         <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1281981468200684</v>
+        <v>6.572227478027344</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9607823558176621</v>
+        <v>0.9100525295165802</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9805194805194806</v>
+        <v>0.9177215189873418</v>
       </c>
       <c r="G3" t="n">
-        <v>0.9745479449394199</v>
+        <v>0.9053970684014629</v>
       </c>
       <c r="H3" t="n">
-        <v>0.9994518468544443</v>
+        <v>0.992708122285623</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>{'metric': 'manhattan', 'n_neighbors': 3, 'weights': 'distance'}</t>
+          <t>{'metric': 'manhattan', 'n_neighbors': 15, 'weights': 'distance'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Classification</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>KNN</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D4" t="n">
+        <v>7.689805746078491</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.9133368902195146</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.9177215189873418</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.9053970684014629</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.992708122285623</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>{'metric': 'manhattan', 'n_neighbors': 15, 'weights': 'distance'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Classification</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>KNN</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>15</v>
+      </c>
+      <c r="D5" t="n">
+        <v>7.842351198196411</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.9129583933927897</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.9177215189873418</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.9053970684014629</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.992708122285623</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>{'metric': 'manhattan', 'n_neighbors': 15, 'weights': 'distance'}</t>
         </is>
       </c>
     </row>

</xml_diff>